<commit_message>
Add Lesson 1.2 Field Log + scrub unassigned regional location
Lesson 1.2 (Soldering Bootcamp) Field Log entry: recap, by-the-numbers,
safety, decisions, action items, what-we-learned, student outcomes, and
looking-ahead. Hero photo published (releases on file) plus a downloadable
one-page PDF. New assets in assets/meetings/1.2/ (3 photos + meeting-note.pdf).
app.js adds hero/safety/outcomes builders and updated render order; style.css
adds hero photo styles.

Remove every asserted "Dauphin Island / DISL / Northern Gulf Coast Regional"
reference — the 2027 regional isn't assigned yet — and replace with neutral
"our 2027 MATE ROV regional (TBD)" phrasing. Covers content.js (calendar,
resources, funding, roadmap, meeting recaps), Bill of Materials (xlsx + pdf),
1.1 Kickoff slides (pptx + pdf), and the regenerated 1.1 meeting-note PDF.

Fix contact email to saywattrobotics2022@gmail.com in both funding blocks.
</commit_message>
<xml_diff>
--- a/Team_Files/Bill of Materials.xlsx
+++ b/Team_Files/Bill of Materials.xlsx
@@ -902,12 +902,12 @@
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>MATE / DISL</t>
+          <t>MATE</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>2027 Northern Gulf Coast Regional</t>
+          <t>2027 regional (assignment TBD)</t>
         </is>
       </c>
       <c r="E7" s="16" t="n">
@@ -942,7 +942,7 @@
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>Dauphin Island, AL — 6 hr drive</t>
+          <t>Travel to our 2027 regional (TBD)</t>
         </is>
       </c>
       <c r="E8" s="16" t="n">

</xml_diff>